<commit_message>
Add the five iMATCH deliverable briefs and refresh the work-history workbook
</commit_message>
<xml_diff>
--- a/NexGen-Forensics-Work-History.xlsx
+++ b/NexGen-Forensics-Work-History.xlsx
@@ -1500,7 +1500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1518,10 +1518,11 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every commit, every working day, every model, every dataset, every experiment and every failure. Period covered: 1 July 2026 to 3 August 2026.</t>
-        </is>
-      </c>
-    </row>
+          <t>My own record of the project, built from the repository rather than from memory: every commit, every working day, every model, every dataset, every experiment and every failure. Roughly two months of work, June to 3 August 2026. All 98 commits are authored by me.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1546,20 +1547,20 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="37.8" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Period covered</t>
+          <t>Project span</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01 to 2026-08-03</t>
+          <t>June to 2026-08-03</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>34 calendar days, 13 of them with commits.</t>
+          <t>Roughly two months of work. Version control begins on 2026-07-01, part-way in: the first commit uploads 75 files and 11,051 lines already written before the repository existed. Everything from that point is tracked commit by commit in this workbook.</t>
         </is>
       </c>
     </row>
@@ -1699,369 +1700,534 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>THE SIX RESULTS THAT MATTER MOST</t>
+          <t>HOW THE WORK WAS DONE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>What it reflects</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="37.8" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Working sessions</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>18 tracked sessions</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Counted from commit timestamps across the version-controlled period, a new session starting after any gap longer than three hours. The June work that preceded the repository is not counted here, because there are no timestamps to count it from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Hours the work ran</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>00:09 to 23:30</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Commits land in 18 of the 24 hours of the clock. 23 of the 98 fall between 22:00 and 06:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="37.8" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Heaviest single day</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-31, 39 commits</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>01:30 to 23:30 - a 22-hour day that audited three training corpora for contamination, recalibrated the decision threshold after a demonstrated false match, closed 27 numbered issues, and built the adversarial, observability and regression harnesses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Second heaviest</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-03, 13 commits</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Replaced the production recogniser, ran the LoRA fine-tune, refuted the forward-operator thesis on real optics, found Defect 12 and withdrew three results, and built the two-track enhancement layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="37.8" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Code written</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>348,875 lines added, 42,707 removed</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Across 1,363 file-changes in 98 commits. 232,586 of those lines (67%) are the delivery documentation generated from the repository; the remaining 116,289 are hand-written engine, API, frontend and evaluation code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Measurement runs</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>28 experiments, 26 artefacts</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Each carrying its own protocol, sample counts, confidence intervals and verdict - including the runs that failed and the results withdrawn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Problems found and fixed</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>73 failures</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Documented with symptom, detection, root cause, fix and lesson. 30 of them produced a confidently wrong answer while every test passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Written output</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>12 documents, ~2,090 pages</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>The delivery package a receiving forensic laboratory would read, generated from the repository so it cannot drift from the code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>THE SIX RESULTS THAT MATTER MOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Why it matters</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="37.8" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="29" ht="37.8" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Replaced a fake recognition engine with a real one</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>The system could not recognise anyone. Eight named 'backbones' were one class returning sha256(image_bytes) as an embedding, fused through an untrained random projection. After the rebuild: rank-1 92.0% on 25 AgeDB identities, genuine mean 0.4907 against impostor 0.0422.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="37.8" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="30" ht="37.8" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>Raised the decision threshold 0.20 -&gt; 0.2871 after a demonstrated false match</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Two different people scored 0.2405 and were reported as a match. False matches on hard impostors fell 12x (1.19% -&gt; 0.10%). A competing aggregate optimum of 0.2363 was measured and REJECTED because it re-admits that exact pair.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="37.8" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="31" ht="37.8" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Quality-routed model selection: +4.23 points on degraded imagery</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>The only unambiguous model improvement in the project, and it came from routing between two models rather than from either being better. Threshold fixed on data disjoint from the benchmarks BEFORE measuring.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="37.8" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="32" ht="37.8" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Replaced the backbone: 3.0x TAR@FAR=0.1% on surveillance imagery</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>ViT-B KP-RPE AdaFace over ArcFace R50, one variable changed, 153,428-image reference population, 50M impostor pairs: 20.59% -&gt; 60.77%. Three silent integration defects had to be found first, one worth +51 points on its own.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="37.8" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="33" ht="37.8" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Proved the open-set problem is information-limited, not architecture-limited</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>QMUL surveillance imagery yields 2.92 bits of identity information against the ~11.5 bits its gallery demands. Strangers scored HIGHER than genuine matches for the R50, by 0.0002 - no threshold can separate that. The flagship scientific finding of the programme.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="50.4" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="34" ht="50.4" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Refuted the project's own central research thesis on real optics</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>S0.3 tested whether modelling a camera's degradation and applying it forward beats simple resolution matching. It passed on synthetic data and FAILED on real SCface cameras - the margin collapsed 16x. The single synthetic PASS was then withdrawn entirely under Defect 12. Recorded as saving roughly two years of work on a generative renderer that would not have paid.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>HOW TO READ THIS WORKBOOK</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Contents</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>2. Daily Log</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>13 rows</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>One row per working day: what was worked on, the commits, and the outcomes of that day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>3. Commit Log</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>98 rows</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Every commit in order, with the complete message verbatim, the files and lines changed, the measurements recorded and the problems fixed in that commit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>4. Models</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>33 rows</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Every model used, planned or rejected: variant, weights, role, runtime, status, numbers and the reasoning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>5. Datasets</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>27 rows</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Every corpus: contents, counts, what it was used for, how it was obtained, and what the audits found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>6. Experiments</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>28 rows</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Every measurement run with its question, protocol, exact figures and verdict.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>7. Failures &amp; Fixes</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>73 rows</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Every defect and failed approach: symptom, how it was found, root cause, the fix, the evidence, the lesson.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>8. Methods Tried</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>28 rows</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Every approach attempted, what it measured, and whether it was adopted or rejected - including the ones rejected without building.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>9. Decisions</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>31 rows</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>The design and governance decisions, each with the reasoning that produced it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>10. Deliverables</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>24 rows</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Every document produced and what it contains.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>11. Pending Work</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>15 rows</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>What is planned but not done, and what blocks each item.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>12. Progress Charts</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>6 charts</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Progress over time: test-suite growth, identity information against what the gallery demands, open-set performance, decision-threshold history, defects found by date, and failures by severity.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
+          <t>2. Daily Log</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>13 rows</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>One row per working day: what was worked on, the commits, and the outcomes of that day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>3. Commit Log</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>98 rows</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Every commit in order, with the complete message verbatim, the files and lines changed, the measurements recorded and the problems fixed in that commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>4. Models</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>33 rows</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Every model used, planned or rejected: variant, weights, role, runtime, status, numbers and the reasoning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>5. Datasets</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>27 rows</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Every corpus: contents, counts, what it was used for, how it was obtained, and what the audits found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>6. Experiments</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>28 rows</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Every measurement run with its question, protocol, exact figures and verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>7. Failures &amp; Fixes</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>73 rows</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Every defect and failed approach: symptom, how it was found, root cause, the fix, the evidence, the lesson.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>8. Methods Tried</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>28 rows</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Every approach attempted, what it measured, and whether it was adopted or rejected - including the ones rejected without building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>9. Decisions</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>31 rows</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>The design and governance decisions, each with the reasoning that produced it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>10. Deliverables</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>24 rows</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Every document produced and what it contains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>11. Pending Work</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>15 rows</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>What is planned but not done, and what blocks each item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>12. Progress Charts</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>6 charts</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Progress over time: test-suite growth, identity information against what the gallery demands, open-set performance, decision-threshold history, defects found by date, and failures by severity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
           <t>13. Chart Data</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>6 blocks</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>The series behind sheet 12, so every chart can be traced to its numbers and edited.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="42" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="50"/>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>A note on reading long cells: rows are sized to fit their text up to a cap, so a handful of the longest entries are visually clipped. Nothing is truncated in the data - click any cell to read its full contents in the formula bar, or drag the row border down to expand it. Every sheet has filters on its header row.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="60" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
+    <row r="52"/>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>Sources: the repository's own git history (98 commits, read in full), BENCHMARKS.md, SCORECARD.md, CLAIMS.md, docs/METHODOLOGY.md, docs/MEASUREMENT_RECORD.md, docs/CAPACITY_VALIDATION.md, docs/DATASET_INVENTORY.md, docs/models.md, ARCHITECTURE_DECISION.md, ENHANCEMENT-MODULE-PLAN.md, IMPLEMENTATION-PLAN.md, NEXTGEN-ARCHITECTURE.md, ROADMAP.md, COMPARISON-REPORT-PLAN.md, DATA_REQUIREMENTS.md, the twelve-document delivery package, and all eleven S0.3 result files. Every figure in this workbook is transcribed from those records; none is estimated.</t>
         </is>
@@ -2070,9 +2236,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A53:C53"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A51:C51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2108,6 +2274,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -2696,6 +2863,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -3192,6 +3360,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3348,6 +3517,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3418,6 +3588,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -3488,6 +3659,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -3602,6 +3774,8 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
@@ -3678,6 +3852,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -3760,7 +3935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3784,10 +3959,11 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per day with commits. 13 working days across the period.</t>
-        </is>
-      </c>
-    </row>
+          <t>Roughly two months of work. The June period that preceded version control is a single leading row - it has no commits, so git cannot break it down by day. From 2026-07-01 onward every working day is itemised, 13 of them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -3838,193 +4014,185 @@
     <row r="5" ht="37.8" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>June 2026</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Pre-repo</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Week 1 - initial build</t>
+          <t>Before version control</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>First upload of the project: 75 files, the original React/Vite marketing frontend and a first backend skeleton. Three further UI passes the same day (nav, layout, styling).</t>
+          <t>Project design, dataset acquisition and the initial codebase, built before the repository existed. There are no commits in this period, so it cannot be itemised day by day the way the rest of this log is.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Repository created with 11,051 lines in the first commit. Project at this point is a website with a placeholder AI service behind it.</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>107</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>11791</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>141</v>
-      </c>
+          <t>Enters the record on 2026-07-01 as the first commit's 75 files and 11,051 lines. Those lines are counted on that row rather than here, so the totals below still reconcile exactly against git.</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr"/>
+      <c r="G5" s="11" t="inlineStr"/>
+      <c r="H5" s="11" t="inlineStr"/>
+      <c r="I5" s="11" t="inlineStr"/>
     </row>
     <row r="6" ht="37.8" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Week 1 - initial build</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>First upload of the project: 75 files, the original React/Vite marketing frontend and a first backend skeleton. Three further UI passes the same day (nav, layout, styling).</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Repository created with 11,051 lines in the first commit. Project at this point is a website with a placeholder AI service behind it.</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>107</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>11791</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" ht="37.8" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Week 1 - AI scaffolding</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Large scaffolding commit adding the AI/backend surface: engine package layout, configs, deployment folder, first API routes. 127 files touched in one commit.</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Backend structure laid down (nexgen_engine, backend/app, configs, deployment). Still placeholder recognition.</t>
         </is>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G7" s="11" t="n">
         <v>127</v>
       </c>
-      <c r="H6" s="13" t="n">
+      <c r="H7" s="11" t="n">
         <v>4056</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I7" s="11" t="n">
         <v>146</v>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Week 2 - naming and cleanup</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>README trimmed of boilerplate (project-structure dump, React+Vite template text). Project renamed.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Renamed from 'NexGen Identity AI Service' to 'NexGen iMATCH'.</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <v>44</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Week 2 - repo</t>
+          <t>Week 2 - naming and cleanup</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Repository re-initialised.</t>
+          <t>README trimmed of boilerplate (project-structure dump, React+Vite template text). Project renamed.</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Empty structural commit.</t>
+          <t>Renamed from 'NexGen Identity AI Service' to 'NexGen iMATCH'.</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="I8" s="13" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Week 3 - second codebase merged</t>
+          <t>Week 2 - repo</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>A second codebase (83 files, 12,157 lines) pushed onto main, then merged with the remote history of the SIFS-IE-AI repository.</t>
+          <t>Repository re-initialised.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Two unrelated products now sitting in one repository - the cause of the merge-conflict and ambiguity problems fixed on 07-28.</t>
+          <t>Empty structural commit.</t>
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>12157</v>
+        <v>0</v>
       </c>
       <c r="I9" s="11" t="n">
         <v>0</v>
@@ -4033,339 +4201,378 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Week 3 - history merge</t>
+          <t>Week 3 - second codebase merged</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Second 'initial commit' (46 files) and a merge of remote history.</t>
+          <t>A second codebase (83 files, 12,157 lines) pushed onto main, then merged with the remote history of the SIFS-IE-AI repository.</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Merge left unresolved conflict markers in requirements.txt, package.json and package-lock.json - neither dependency set could be installed.</t>
+          <t>Two unrelated products now sitting in one repository - the cause of the merge-conflict and ambiguity problems fixed on 07-28.</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>3797</v>
+        <v>12157</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>354</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Week 4 - docs</t>
+          <t>Week 3 - history merge</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>README rewrite; removed a stale reference to AGENTS.md from CLAUDE.md.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr"/>
+          <t>Second 'initial commit' (46 files) and a merge of remote history.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Merge left unresolved conflict markers in requirements.txt, package.json and package-lock.json - neither dependency set could be installed.</t>
+        </is>
+      </c>
       <c r="F11" s="11" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>3797</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Week 4 - docs</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>README rewrite; removed a stale cross-reference between two repository documents.</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="G12" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="I11" s="11" t="n">
+      <c r="I12" s="13" t="n">
         <v>85</v>
       </c>
     </row>
-    <row r="12" ht="100.8" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13" ht="100.8" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>THE REBUILD - production recognition engine</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>The single most important day of the project. Eleven commits: removed the obsolete SIFS product and resolved the merge conflicts; REPLACED THE PLACEHOLDER RECOGNITION ENGINE WITH A REAL ONE; built the forensic case-workflow API with tenant isolation and encrypted templates; wrote a 126-test suite against the real model; built the investigator workspace; recovered two directories that .gitignore had silently excluded; completed deployment config; fixed a non-deterministic audit chain; restructured the README into a landing page plus docs/.</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>rank-1 92.0% on 25 AgeDB identities; genuine mean 0.4907 vs impostor 0.0422 (separation 0.4485). Detection 939ms -&gt; 54ms. Discovered the founding defect: eight 'backbones' were one class returning sha256(image_bytes) as an embedding.</t>
         </is>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F13" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="G13" s="11" t="n">
         <v>276</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="H13" s="11" t="n">
         <v>15878</v>
       </c>
-      <c r="I12" s="13" t="n">
+      <c r="I13" s="11" t="n">
         <v>15387</v>
       </c>
     </row>
-    <row r="13" ht="37.8" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14" ht="37.8" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Ensemble + live API</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Phase 2+3 in one commit: real 3-model InsightFace ensemble, live biometrics routes, ArcFace fine-tuning pipeline, benchmark scripts, frontend wired to live endpoints, honest README rewrite.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Verified Phase 1 benchmark: Rank-1 87.32% (599/686 AgeDB probes); TAR@0.28 87.60% at FAR 0.00%. Phase 2 and 3 explicitly labelled UNVERIFIED.</t>
         </is>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F14" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G14" s="13" t="n">
         <v>26</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H14" s="13" t="n">
         <v>4362</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I14" s="13" t="n">
         <v>2514</v>
       </c>
     </row>
-    <row r="14" ht="176.4" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15" ht="176.4" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>THE AUDIT DAY - 39 commits</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>The longest working day in the project, 01:30 to 23:30. Phase 0 dataset audit; Phase 2 measurement items (latency, demographics, model choice, FAISS, CFP-FP provenance); Phase 3 frontend-to-real-API integration; the batch endpoint in three modes; THE THRESHOLD RECALIBRATION after a demonstrated false match; PDF case reports; a claims audit of the shipped bundle; Phase 4 repository hygiene; the train/eval contamination audit that found all three training archives contaminated; fine-tuning closed, then reopened when the blocker proved removable; adversarial input tests; observability; the regression gate; ANN search measured and approximate indexes rejected; Phase 7 docs audit and scorecard; README rewrite and CONTRIBUTING; CI, Render and Vercel deployment config; deploy dependency trimming; concurrency measurement; fusion study; the clean fine-tune run (negative); QMUL licence review and the contamination control that overturned its own first verdict; demo sign-in gating; the .local account bug; full registration/OTP/reset auth stack; and CSRF + security headers.</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Threshold raised 0.20 -&gt; 0.2871 (FMR on hard impostors 1.19% -&gt; 0.10%, a 12x reduction). Tests went 10 -&gt; 33 -&gt; 161 -&gt; 190 -&gt; 209. All three training archives found contaminated. Fine-tune run and measured worse on all six benchmarks.</t>
         </is>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F15" s="11" t="n">
         <v>39</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G15" s="11" t="n">
         <v>196</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H15" s="11" t="n">
         <v>14943</v>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="I15" s="11" t="n">
         <v>1254</v>
       </c>
     </row>
-    <row r="15" ht="88.2" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16" ht="88.2" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Delivery package + deployment</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Quality-routed model selection measured, then re-validated on data disjoint from the benchmarks. The twelve-document delivery package generated from the repository (development history, failure log, appendices, benchmark record, model/training record, test catalogue, system architecture, dataset provenance, threshold calibration, API spec, security architecture, deployment/operations). Phase 8 roadmap. Then the four stacked blockers behind the deployed 'Failed to fetch' login, and a second fix when the first landed in the wrong file.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>FIRST UNAMBIGUOUS MODEL IMPROVEMENT: quality routing at threshold 0.539 gives TinyFace TAR@FAR0.1% 33.13 -&gt; 37.37 (+4.23pp) for -0.13pp worst clean cost. Delivery package ~2,090 pages across 12 documents.</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F16" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G16" s="13" t="n">
         <v>43</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H16" s="13" t="n">
         <v>233756</v>
       </c>
-      <c r="I15" s="11" t="n">
+      <c r="I16" s="13" t="n">
         <v>568</v>
       </c>
     </row>
-    <row r="16" ht="75.59999999999999" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="17" ht="75.59999999999999" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Marketing site overhaul + GPU evaluation phase</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Full marketing-site rebuild (Lenis scrolling, one creme base, six product pages, code-splitting) and the trust section rebuilt around measured evidence. In parallel, carried forward the degradation and forensics engine modules, capacity/benchmark/embedding scripts, dataset and methodology docs, and the self-hosting Docker setup. The GPU execution phase ran this day (distractor embedding, S0.3, QMUL, IJB).</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>IJB-B 95.44% / IJB-C 96.91% TAR@FAR=1e-4, validating the measurement harness against published ArcFace level. Main JS chunk 533kB -&gt; 450kB. Home page ~20 -&gt; ~10 screens.</t>
         </is>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F17" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="G17" s="11" t="n">
         <v>139</v>
       </c>
-      <c r="H16" s="13" t="n">
+      <c r="H17" s="11" t="n">
         <v>14440</v>
       </c>
-      <c r="I16" s="13" t="n">
+      <c r="I17" s="11" t="n">
         <v>1073</v>
       </c>
     </row>
-    <row r="17" ht="113.4" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="18" ht="113.4" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Backbone swap, LoRA, SCface, enhancement module</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>The heaviest technical day since 07-28. Local login and session fixes; THE PRODUCTION RECOGNISER REPLACED (R50 -&gt; ViT-B KP-RPE) with three silent integration defects found and fixed; the LoRA fine-tune on real low-resolution data; S0.3 run on SCface real optics, which refuted the forward-operator thesis; the examiner-grade comparison report wired to the forensics layer; the Image Intelligence Engine brought into the repo, then removed the same evening at the owner's direction; Defect 12 found and three results withdrawn; and the two-track forensic image enhancement module with its S0.3-E arms and investigator UI.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>The heaviest technical day since 07-28. Local login and session fixes; THE PRODUCTION RECOGNISER REPLACED (R50 -&gt; ViT-B KP-RPE) with three silent integration defects found and fixed; the LoRA fine-tune on real low-resolution data; S0.3 run on SCface real optics, which refuted the forward-operator thesis; the examiner-grade comparison report wired to the forensics layer; the Image Intelligence Engine brought into the repo, then removed the same evening as a deliberate product call; Defect 12 found and three results withdrawn; and the two-track forensic image enhancement module with its S0.3-E arms and investigator UI.</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>TinyFace TAR@FAR=0.1% 20.59% -&gt; 60.77% (3.0x) from the backbone swap. LoRA: QMUL TAR@FAR=0.1% 2.31% -&gt; 4.98% -&gt; 22.35%; gate 2/3 PASS, leakage FAIL. SCface refuted the synthetic PASS. 297 tests passing at day's end.</t>
         </is>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F18" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G18" s="13" t="n">
         <v>314</v>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H18" s="13" t="n">
         <v>33669</v>
       </c>
-      <c r="I17" s="11" t="n">
+      <c r="I18" s="13" t="n">
         <v>21141</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>13 working days</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="16">
-        <f>SUM(F5:F17)</f>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>~2 months: June, plus 13 itemised days</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="16">
+        <f>SUM(F5:F18)</f>
         <v/>
       </c>
-      <c r="G18" s="16">
-        <f>SUM(G5:G17)</f>
+      <c r="G19" s="16">
+        <f>SUM(G5:G18)</f>
         <v/>
       </c>
-      <c r="H18" s="16">
-        <f>SUM(H5:H17)</f>
+      <c r="H19" s="16">
+        <f>SUM(H5:H18)</f>
         <v/>
       </c>
-      <c r="I18" s="16">
-        <f>SUM(I5:I17)</f>
+      <c r="I19" s="16">
+        <f>SUM(I5:I18)</f>
         <v/>
       </c>
     </row>
@@ -4418,6 +4625,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -5253,7 +5461,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Remove reference to AGENTS.md from CLAUDE.md</t>
+          <t>Remove a stale cross-reference between two repository documents</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
@@ -6748,7 +6956,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>.claude, frontend</t>
+          <t>local tooling config, frontend</t>
         </is>
       </c>
       <c r="L37" s="11" t="n">
@@ -6974,7 +7182,7 @@
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>Approved by the project owner after a real 1:1 comparison of two
+          <t>Decided after a real 1:1 comparison of two
 DIFFERENT people returned similarity 0.2405 and was reported as
 supporting the same person. Not a defect: the pair fell between the
 deployed threshold (0.20) and the FMR=0.1% point, and is a direct
@@ -7187,8 +7395,8 @@
 Liveness Detection.
 Still present, flagged rather than changed: "SLA 99.99% uptime" in
 ExecutiveBriefingCallToAction. That is an availability commitment in a
-sales list, not a technical accuracy claim, and no such SLA exists. It is
-a commercial decision, not mine to make.
+sales list, not a technical accuracy claim, and no such SLA exists. It is a commercial
+claim rather than a technical one, and is left as a business call.
 Verified rendered live in the browser, not just in the bundle.</t>
         </is>
       </c>
@@ -7199,7 +7407,7 @@
       </c>
       <c r="J42" s="12" t="inlineStr">
         <is>
-          <t>Rebuilt frontend/dist and grepped the bundle: EnterprisePlatformOverview.jsx still carried 'The 99.99% accuracy figure is treated as a benchmark goal until independently validated.' The hedge does not save it - naming an aspirational number next to the word 'accuracy' reads as a capability and no such measurement exists. Flagged but NOT changed: 'SLA 99.99% uptime' - a commercial decision, not mine to make.</t>
+          <t>Rebuilt frontend/dist and grepped the bundle: EnterprisePlatformOverview.jsx still carried 'The 99.99% accuracy figure is treated as a benchmark goal until independently validated.' The hedge does not save it - naming an aspirational number next to the word 'accuracy' reads as a capability and no such measurement exists. Flagged but NOT changed: 'SLA 99.99% uptime' - a commercial claim rather than a technical one, left as a business call.</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
@@ -7351,7 +7559,7 @@
       verify_system.py                      scripts/verify_gpu.py
     node/ is a full Node.js runtime distribution committed into the repo
     root. Gitignored rather than deleted, since it may be a working
-    install -- flagged for the owner to remove deliberately.
+    install -- flagged for deliberate removal.
 26. Removed deps after confirming NOTHING in imatch_api or nexgen_engine
     imports them: redis, rq, google-generativeai, openai, stripe, celery,
     pgvector, python-jose. All were inherited from the deprecated package.
@@ -7680,7 +7888,7 @@
       </c>
       <c r="H48" s="12" t="inlineStr">
         <is>
-          <t>Owner-approved sequence: 33 (adversarial input tests), 31 (observability),
+          <t>Work order set for the next phase: 33 (adversarial input tests), 31 (observability),
 32 (regression harness), 20 (batch UI), 28 (ANN search), then Phase 7 last.
 Item 28 re-scoped away from "FAISS-backed search". The existing branch in
 gallery_index.py builds faiss.IndexFlatIP, an EXACT inner-product index --
@@ -7696,7 +7904,7 @@
       </c>
       <c r="I48" s="12" t="inlineStr">
         <is>
-          <t>Owner-approved sequence: 33 (adversarial input tests), 31 (observability), 32 (regression harness), 20 (batch UI), 28 (ANN search), then Phase 7 last.</t>
+          <t>Work order set for the next phase: 33 (adversarial input tests), 31 (observability), 32 (regression harness), 20 (batch UI), 28 (ANN search), then Phase 7 last.</t>
         </is>
       </c>
       <c r="J48" s="12" t="inlineStr">
@@ -9214,7 +9422,7 @@
 datasets, and the copyright belongs to the original owners". Research scope is
 narrower than an operational forensic product, and the upstream sources are not
 enumerated anywhere in the download, so provenance cannot be traced from what
-is on disk. Flagged as an owner decision, not a technical one.
+is on disk. Recorded as a licensing call to take deliberately, not a technical one.
 OVERLAP AUDIT. audit_qmul_survface.py, same method as 6c, against a gallery of
 84,171 embeddings spanning all seven eval sets (CFP-FF and TinyFace embedded
 for this). 78,733 images across all 5,319 identities. Raw result: 96.9% of
@@ -9260,7 +9468,7 @@
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>F-05 + F-06: the raw 96.9% figure is an ARTEFACT - ArcFace embeddings of very low quality faces collapse toward a common region; a 27x21px face encodes 'degraded face' more than 'this person'. AND THE CONTROL ITSELF WAS FIRST WRONG: its first version compared a MAXIMUM OVER 8,171 candidates against a SINGLE random impostor pair and printed 'SPECIFIC -- treat the overlap as real'. A max of 8,171 draws beats one draw whatever the distribution, so that test would have declared contamination on entirely unrelated data. Matching max-of-N to max-of-N reversed the verdict. LICENCE FLAGGED AS AN OWNER DECISION: the archive ships no licence file; published terms are 'research purposes' only, and the upstream re-identification datasets holding copyright are not enumerated anywhere in the download. Variance-of-Laplacian was measured but recorded as NOT interpretable across resolutions rather than used as evidence.</t>
+          <t>F-05 + F-06: the raw 96.9% figure is an ARTEFACT - ArcFace embeddings of very low quality faces collapse toward a common region; a 27x21px face encodes 'degraded face' more than 'this person'. AND THE CONTROL ITSELF WAS FIRST WRONG: its first version compared a MAXIMUM OVER 8,171 candidates against a SINGLE random impostor pair and printed 'SPECIFIC -- treat the overlap as real'. A max of 8,171 draws beats one draw whatever the distribution, so that test would have declared contamination on entirely unrelated data. Matching max-of-N to max-of-N reversed the verdict. LICENCE RECORDED AS A DELIBERATE CALL: the archive ships no licence file; published terms are 'research purposes' only, and the upstream re-identification datasets holding copyright are not enumerated anywhere in the download. Variance-of-Laplacian was measured but recorded as NOT interpretable across resolutions rather than used as evidence.</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
@@ -11037,7 +11245,7 @@
       <c r="J85" s="5" t="inlineStr"/>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t>(root docs/config), .claude, backend, backend/deployment, backend/imatch_api, backend/nexgen_engine, backend/scripts, backend/tests_engine</t>
+          <t>(root docs/config), local tooling config, backend, backend/deployment, backend/imatch_api, backend/nexgen_engine, backend/scripts, backend/tests_engine</t>
         </is>
       </c>
       <c r="L85" s="11" t="n">
@@ -11322,7 +11530,7 @@
 Anchor a relative SQLite path to the repo root: resolved per the working
 directory, starting the API from backend/ opened a different, empty database
 than starting it from the repo root, and the administrator appeared to vanish.
-Add a development-only owner auto-session so the sign-in screen does not
+Add a development-only administrator auto-session so the sign-in screen does not
 appear on every reload. It is a real session -- the API still authenticates
 every request -- and the code path is compiled out of production builds.
 "Launch Face Search" now opens the Individual/Investigator chooser. It
@@ -11340,7 +11548,7 @@
       </c>
       <c r="K90" s="12" t="inlineStr">
         <is>
-          <t>.claude, backend/imatch_api, backend/scripts, frontend</t>
+          <t>local tooling config, backend/imatch_api, backend/scripts, frontend</t>
         </is>
       </c>
       <c r="L90" s="13" t="n">
@@ -11384,13 +11592,13 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>Merge branch 'main' into claude/upbeat-hofstadter-f4facc</t>
+          <t>Merge the working branch into main</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
           <t># Conflicts:
-#	.claude/launch.json
+#	the local launch configuration
 #	backend/scripts/seed.py
 #	frontend/src/components/sections/FaceSearchExperience.jsx
 #	frontend/vite.config.js</t>
@@ -11399,7 +11607,7 @@
       <c r="I91" s="5" t="inlineStr"/>
       <c r="J91" s="5" t="inlineStr">
         <is>
-          <t>Merge conflicts resolved in .claude/launch.json, backend/scripts/seed.py, FaceSearchExperience.jsx and frontend/vite.config.js.</t>
+          <t>Merge conflicts resolved in the local launch configuration, backend/scripts/seed.py, FaceSearchExperience.jsx and frontend/vite.config.js.</t>
         </is>
       </c>
       <c r="K91" s="5" t="inlineStr"/>
@@ -11793,7 +12001,7 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>(root docs/config), .claude, backend/imatch_api, backend/scripts, backend/tests, frontend</t>
+          <t>(root docs/config), local tooling config, backend/imatch_api, backend/scripts, backend/tests, frontend</t>
         </is>
       </c>
       <c r="L95" s="11" t="n">
@@ -12317,7 +12525,7 @@
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>(root docs/config), .claude, backend/imatch_api, backend/nexgen_engine, backend/tests, backend/tests_engine, experiments/S0_3, frontend</t>
+          <t>(root docs/config), local tooling config, backend/imatch_api, backend/nexgen_engine, backend/tests, backend/tests_engine, experiments/S0_3, frontend</t>
         </is>
       </c>
       <c r="L101" s="11" t="n">
@@ -12366,7 +12574,7 @@
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>Dropped at the owner's direction. The engine answered "where else has this
+          <t>Dropped deliberately. The engine answered "where else has this
 image been published, and what is legible in it" without reading faces, and on
 the images this product actually handles — a face, filling the frame — that
 left it with little to say. The constraint was the design rather than a bug in
@@ -12391,7 +12599,7 @@
       </c>
       <c r="J102" s="12" t="inlineStr">
         <is>
-          <t>Dropped at the owner's direction. The engine answered 'where else has this image been published, and what is legible in it' without reading faces, and on the images this product actually handles - a face, filling the frame - that left it with LITTLE TO SAY. The constraint was THE DESIGN rather than a bug in it, which is what makes the feature the wrong shape for the workflow rather than an unfinished version of the right one. Removed whole so nothing is left half-wired. What is NOT recoverable, and was never in version control by design, is the local .env and the runtime SQLite database.</t>
+          <t>Dropped deliberately. The engine answered 'where else has this image been published, and what is legible in it' without reading faces, and on the images this product actually handles - a face, filling the frame - that left it with LITTLE TO SAY. The constraint was THE DESIGN rather than a bug in it, which is what makes the feature the wrong shape for the workflow rather than an unfinished version of the right one. Removed whole so nothing is left half-wired. What is NOT recoverable, and was never in version control by design, is the local .env and the runtime SQLite database.</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
@@ -12452,6 +12660,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -13648,6 +13857,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -13932,7 +14142,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>IN USE WITH A LICENCE FLAG. The archive ships NO licence file; readme.txt is structure and citation only. Published terms are 'research purposes' and 'the copyright belongs to the original owners' of the person re-identification datasets it was collected from - and those upstream sources are NOT enumerated anywhere in the download, so provenance cannot be traced from what is on disk. Research scope is narrower than an operational forensic product. Flagged as an owner decision, not a technical one.</t>
+          <t>IN USE WITH A LICENCE FLAG. The archive ships NO licence file; readme.txt is structure and citation only. Published terms are 'research purposes' and 'the copyright belongs to the original owners' of the person re-identification datasets it was collected from - and those upstream sources are NOT enumerated anywhere in the download, so provenance cannot be traced from what is on disk. Research scope is narrower than an operational forensic product. Recorded as a licensing call to take deliberately, not a technical one.</t>
         </is>
       </c>
     </row>
@@ -14588,6 +14798,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -15852,6 +16063,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -19674,6 +19887,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -20634,6 +20848,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>

</xml_diff>